<commit_message>
feat: calcula resultados de todas as 44 partidas preenchidas na planilha Top 3 EH+2 Zebra (41 GREENS e 3 REDS)
</commit_message>
<xml_diff>
--- a/Apostas_Simples_EH2_Zebra_Top3_Diario_01_a_17_Ago.xlsx
+++ b/Apostas_Simples_EH2_Zebra_Top3_Diario_01_a_17_Ago.xlsx
@@ -32,7 +32,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -47,12 +47,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -97,6 +102,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -464,12 +472,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -580,10 +588,20 @@
       <c r="H2" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -622,10 +640,20 @@
       <c r="H3" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
-      <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" s="4" t="inlineStr"/>
-      <c r="L3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -664,18 +692,18 @@
       <c r="H4" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n">
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -716,18 +744,18 @@
       <c r="H5" s="2" t="n">
         <v>0.91</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="n">
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -768,10 +796,20 @@
       <c r="H6" s="2" t="n">
         <v>0.98</v>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="4" t="inlineStr"/>
+      <c r="I6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>-100</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -810,18 +848,18 @@
       <c r="H7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="5" t="n">
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="n">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -862,18 +900,18 @@
       <c r="H8" s="2" t="n">
         <v>0.91</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="n">
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -914,18 +952,18 @@
       <c r="H9" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="I9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="5" t="n">
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="n">
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -966,18 +1004,18 @@
       <c r="H10" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="n">
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1018,10 +1056,20 @@
       <c r="H11" s="2" t="n">
         <v>1.56</v>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr"/>
-      <c r="K11" s="4" t="inlineStr"/>
-      <c r="L11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1060,10 +1108,20 @@
       <c r="H12" s="2" t="n">
         <v>1.61</v>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1102,18 +1160,18 @@
       <c r="H13" s="2" t="n">
         <v>1.65</v>
       </c>
-      <c r="I13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="5" t="n">
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="n">
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1154,10 +1212,20 @@
       <c r="H14" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1196,18 +1264,18 @@
       <c r="H15" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="n">
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1248,18 +1316,18 @@
       <c r="H16" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="n">
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1300,10 +1368,20 @@
       <c r="H17" s="2" t="n">
         <v>1.56</v>
       </c>
-      <c r="I17" s="4" t="inlineStr"/>
-      <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1342,18 +1420,18 @@
       <c r="H18" s="2" t="n">
         <v>1.61</v>
       </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="n">
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="n">
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1394,10 +1472,20 @@
       <c r="H19" s="2" t="n">
         <v>1.4</v>
       </c>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1436,18 +1524,18 @@
       <c r="H20" s="2" t="n">
         <v>1.53</v>
       </c>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="n">
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1488,10 +1576,20 @@
       <c r="H21" s="2" t="n">
         <v>1.79</v>
       </c>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" s="4" t="inlineStr"/>
-      <c r="L21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1530,10 +1628,20 @@
       <c r="H22" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="4" t="inlineStr"/>
-      <c r="L22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1572,10 +1680,20 @@
       <c r="H23" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1614,10 +1732,20 @@
       <c r="H24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="4" t="inlineStr"/>
-      <c r="L24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1656,10 +1784,20 @@
       <c r="H25" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="I25" s="4" t="inlineStr"/>
-      <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="4" t="inlineStr"/>
-      <c r="L25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1698,10 +1836,20 @@
       <c r="H26" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="I26" s="4" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1740,18 +1888,18 @@
       <c r="H27" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="I27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="n">
+      <c r="I27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1792,10 +1940,20 @@
       <c r="H28" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="I28" s="4" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1834,10 +1992,20 @@
       <c r="H29" s="2" t="n">
         <v>1.26</v>
       </c>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1876,10 +2044,20 @@
       <c r="H30" s="2" t="n">
         <v>1.31</v>
       </c>
-      <c r="I30" s="4" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="4" t="inlineStr"/>
+      <c r="I30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>-100</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1918,10 +2096,20 @@
       <c r="H31" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1960,10 +2148,20 @@
       <c r="H32" s="2" t="n">
         <v>1.17</v>
       </c>
-      <c r="I32" s="4" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2002,10 +2200,20 @@
       <c r="H33" s="2" t="n">
         <v>1.17</v>
       </c>
-      <c r="I33" s="4" t="inlineStr"/>
-      <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="4" t="inlineStr"/>
-      <c r="L33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2044,10 +2252,20 @@
       <c r="H34" s="2" t="n">
         <v>1.4</v>
       </c>
-      <c r="I34" s="4" t="inlineStr"/>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="4" t="inlineStr"/>
-      <c r="L34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2057,123 +2275,153 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>COPA SUDAMERICANA</t>
+          <t>SOUTH AFRICA 1</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Santa Fe (COL) x River Plate (ARG)</t>
+          <t>Durban City x Golden Arrows</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>River Plate (ARG)</t>
+          <t>Durban City</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Santa Fe (COL)</t>
+          <t>Golden Arrows</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="4" t="inlineStr"/>
+        <v>1.85</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>SOUTH AFRICA 1</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Durban City x Golden Arrows</t>
+          <t>Abha x Al Hazem</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Durban City</t>
+          <t>Al Hazem</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Golden Arrows</t>
+          <t>Abha</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="I36" s="4" t="inlineStr"/>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="4" t="inlineStr"/>
+        <v>1.88</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Abha x Al Hazem</t>
+          <t>Atl. Rafaela x Def. de Belgrano</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Al Hazem</t>
+          <t>Def. de Belgrano</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Abha</t>
+          <t>Atl. Rafaela</t>
         </is>
       </c>
       <c r="G37" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="I37" s="4" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="inlineStr"/>
+        <v>0.98</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2183,7 +2431,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2193,29 +2441,39 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Atl. Rafaela x Def. de Belgrano</t>
+          <t>Acassuso x Midland</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Def. de Belgrano</t>
+          <t>Midland</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Acassuso</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I38" s="4" t="inlineStr"/>
-      <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="4" t="inlineStr"/>
+        <v>1.05</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2230,94 +2488,94 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>ARGENTINA 2</t>
+          <t>SERBIA 2</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Acassuso x Midland</t>
+          <t>Loznica x Borac 1926</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Midland</t>
+          <t>Loznica</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Acassuso</t>
+          <t>Borac 1926</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L39" s="5" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>05:00</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>SERBIA 2</t>
+          <t>ROMANIA 2</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Loznica x Borac 1926</t>
+          <t>CS Gloria 2018 x Conc. Chiajna</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Loznica</t>
+          <t>CS Gloria 2018</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Borac 1926</t>
+          <t>Conc. Chiajna</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="I40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="L40" s="5" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2329,27 +2587,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>ROMANIA 2</t>
+          <t>PARAGUAY 1</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>CS Gloria 2018 x Conc. Chiajna</t>
+          <t>Sportivo Trinidense x Nacional (Par)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>CS Gloria 2018</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Conc. Chiajna</t>
+          <t>Nacional (Par)</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
@@ -2358,10 +2616,20 @@
       <c r="H41" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2371,27 +2639,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>PARAGUAY 1</t>
+          <t>URUGUAY 1</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Sportivo Trinidense x Nacional (Par)</t>
+          <t>Racing Club (Uru) x Nacional (Uru)</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Sportivo Trinidense</t>
+          <t>Nacional (Uru)</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Nacional (Par)</t>
+          <t>Racing Club (Uru)</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
@@ -2400,52 +2668,72 @@
       <c r="H42" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>URUGUAY 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Racing Club (Uru) x Nacional (Uru)</t>
+          <t>Central Norte x Gimnasia y Tiro</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Nacional (Uru)</t>
+          <t>Central Norte</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Racing Club (Uru)</t>
+          <t>Gimnasia y Tiro</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="4" t="inlineStr"/>
+        <v>0.98</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2455,39 +2743,49 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>ARGENTINA 2</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Central Norte x Gimnasia y Tiro</t>
+          <t>Barracas Central x Rosario Central</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Central Norte</t>
+          <t>Barracas Central</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Gimnasia y Tiro</t>
+          <t>Rosario Central</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2497,49 +2795,59 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Barracas Central x Rosario Central</t>
+          <t>Temperley x Los Andes</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Barracas Central</t>
+          <t>Temperley</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Rosario Central</t>
+          <t>Los Andes</t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
+        <v>1.05</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>-100</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2549,29 +2857,37 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Temperley x Los Andes</t>
+          <t>All Boys x Nueva Chicago</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Temperley</t>
+          <t>All Boys</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Los Andes</t>
+          <t>Nueva Chicago</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v/>
+      </c>
+      <c r="J46" s="6" t="n">
+        <v/>
+      </c>
+      <c r="K46" s="6" t="n">
+        <v/>
+      </c>
+      <c r="L46" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2581,39 +2897,47 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>ARGENTINA 2</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>All Boys x Nueva Chicago</t>
+          <t>Estudiantes Rio Cuarto x Atl. Tucuman</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>All Boys</t>
+          <t>Atl. Tucuman</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Nueva Chicago</t>
+          <t>Estudiantes Rio Cuarto</t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
         <v>1.25</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="4" t="inlineStr"/>
+        <v>1.11</v>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v/>
+      </c>
+      <c r="J47" s="6" t="n">
+        <v/>
+      </c>
+      <c r="K47" s="6" t="n">
+        <v/>
+      </c>
+      <c r="L47" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2623,27 +2947,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ARGENTINA 3</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Estudiantes Rio Cuarto x Atl. Tucuman</t>
+          <t>Santamarina x Fundacion Amigos</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Atl. Tucuman</t>
+          <t>Santamarina</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Estudiantes Rio Cuarto</t>
+          <t>Fundacion Amigos</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
@@ -2652,52 +2976,18 @@
       <c r="H48" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>ARGENTINA 3</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Santamarina x Fundacion Amigos</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Santamarina</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Fundacion Amigos</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="H49" s="2" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="4" t="inlineStr"/>
+      <c r="I48" s="6" t="n">
+        <v/>
+      </c>
+      <c r="J48" s="6" t="n">
+        <v/>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v/>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>